<commit_message>
Entrega final 14/10: robo e linhas do William revisados, 383 precos
</commit_message>
<xml_diff>
--- a/_historico/merge/candidatos.xlsx
+++ b/_historico/merge/candidatos.xlsx
@@ -1319,6 +1319,11 @@
           <t>49.4</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>52.00</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr">
         <is>
           <t>74.85</t>
@@ -1336,7 +1341,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -1478,6 +1483,11 @@
           <t>113.88</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>117.40</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
           <t>36.1</t>
@@ -1495,7 +1505,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1890,12 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>REPROVADO</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Produto não corresponde: a descrição diz "Comprimento: 26cm" (cano curto); o insumo pede cano médio ou longo (decisão de 14/10/2026)</t>
         </is>
       </c>
     </row>
@@ -3227,6 +3242,11 @@
           <t>16.9</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>16.10</t>
+        </is>
+      </c>
       <c r="N35" t="inlineStr">
         <is>
           <t>frete nao calculado: fornecedor com sede em GO</t>
@@ -3239,7 +3259,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -3316,7 +3336,12 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>REPROVADO</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Print reduzido: nome, preço e frete ilegíveis</t>
         </is>
       </c>
     </row>
@@ -3393,7 +3418,12 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>REPROVADO</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Frete coberto pelo banner de cookies no print</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3500,12 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>REPROVADO</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Nome do produto encoberto pelo menu do site no print</t>
         </is>
       </c>
     </row>
@@ -3542,7 +3577,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -4096,7 +4131,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -5900,7 +5935,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6176,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -10216,7 +10251,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -11185,7 +11220,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -11426,7 +11461,7 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -13861,7 +13896,7 @@
       </c>
       <c r="P166" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -14020,7 +14055,12 @@
       </c>
       <c r="P168" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>REPROVADO</t>
+        </is>
+      </c>
+      <c r="Q168" t="inlineStr">
+        <is>
+          <t>CEP não preenchido: frete não aparece no print</t>
         </is>
       </c>
     </row>
@@ -16219,7 +16259,7 @@
       </c>
       <c r="P195" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -16296,7 +16336,12 @@
       </c>
       <c r="P196" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>REPROVADO</t>
+        </is>
+      </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>Produto não corresponde: papel higiênico interfolhado (cai-cai), sem rolo; o insumo pede metragem por rolo (decisão de 14/10/2026)</t>
         </is>
       </c>
     </row>
@@ -18567,7 +18612,12 @@
       </c>
       <c r="P224" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>REPROVADO</t>
+        </is>
+      </c>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>Produto não corresponde: sabonete antisséptico "Sem Aroma" (rótulo); o insumo é sabonete com fragrância</t>
         </is>
       </c>
     </row>
@@ -21740,7 +21790,7 @@
       </c>
       <c r="P263" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -24637,7 +24687,7 @@
       </c>
       <c r="P299" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -25455,6 +25505,11 @@
           <t>1114.44</t>
         </is>
       </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>1173.10</t>
+        </is>
+      </c>
       <c r="M309" t="inlineStr">
         <is>
           <t>236.52</t>
@@ -25472,7 +25527,7 @@
       </c>
       <c r="P309" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -30365,7 +30420,12 @@
       </c>
       <c r="P368" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>REPROVADO</t>
+        </is>
+      </c>
+      <c r="Q368" t="inlineStr">
+        <is>
+          <t>Produto não corresponde: lavadora para serviços domésticos (descrição da página); o insumo é de uso profissional</t>
         </is>
       </c>
     </row>
@@ -30673,7 +30733,7 @@
       </c>
       <c r="P372" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -34286,7 +34346,12 @@
       </c>
       <c r="P416" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>REPROVADO</t>
+        </is>
+      </c>
+      <c r="Q416" t="inlineStr">
+        <is>
+          <t>Print só mostra o preço com desconto ("Por R$ 32,87" com 5% no boleto/PIX já aplicado); o preço lido (40,71) é o "De" riscado</t>
         </is>
       </c>
     </row>
@@ -34363,7 +34428,7 @@
       </c>
       <c r="P417" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>
@@ -34505,6 +34570,11 @@
           <t>55.81</t>
         </is>
       </c>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t>55.81</t>
+        </is>
+      </c>
       <c r="M419" t="inlineStr">
         <is>
           <t>20.49</t>
@@ -34522,7 +34592,7 @@
       </c>
       <c r="P419" t="inlineStr">
         <is>
-          <t>A REVISAR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>

</xml_diff>